<commit_message>
added card rarity probability
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/dev/Raising.xlsx
+++ b/Assets/StreamingAssets/Configurations/dev/Raising.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F897CB7-53D5-4F1C-BE4C-F48006164CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0910DFD-BBE2-466F-ABC6-D09555C637AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RaisingEffects" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="213">
   <si>
     <t>ID</t>
   </si>
@@ -735,6 +735,12 @@
   </si>
   <si>
     <t>4,2,4</t>
+  </si>
+  <si>
+    <t>0.5,0.3,0.2,0.8,0.2,0.1</t>
+  </si>
+  <si>
+    <t>0.2,0.7,0.1,0.8,0.2,0.1</t>
   </si>
 </sst>
 </file>
@@ -1342,6 +1348,9 @@
       <c r="E10">
         <v>0</v>
       </c>
+      <c r="F10" t="s">
+        <v>211</v>
+      </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11">
@@ -1606,7 +1615,10 @@
         <v>60</v>
       </c>
       <c r="E26">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="F26" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="27" spans="1:6">

</xml_diff>

<commit_message>
added 2 attributes on ui
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/dev/Raising.xlsx
+++ b/Assets/StreamingAssets/Configurations/dev/Raising.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0910DFD-BBE2-466F-ABC6-D09555C637AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{082EB76E-5EC7-48BC-BE66-8FA2D9CEF6B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RaisingEffects" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
simplified dialogue loading process
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/dev/Raising.xlsx
+++ b/Assets/StreamingAssets/Configurations/dev/Raising.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39A8CDBA-30F2-46A9-8EF4-4295D259CCA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F3842F3-39F8-45FF-BF77-C58575B1E9F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RaisingEffects" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="212">
   <si>
     <t>ID</t>
   </si>
@@ -729,6 +729,15 @@
   </si>
   <si>
     <t>add coop value for goomba</t>
+  </si>
+  <si>
+    <t>test1</t>
+  </si>
+  <si>
+    <t>Graduation_3</t>
+  </si>
+  <si>
+    <t>Graduation_4</t>
   </si>
 </sst>
 </file>
@@ -1939,8 +1948,8 @@
       <c r="I2" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="K2" s="3">
-        <v>0</v>
+      <c r="K2" s="3" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="30" customHeight="1">
@@ -1971,8 +1980,8 @@
       <c r="I3" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="K3" s="3">
-        <v>0</v>
+      <c r="K3" s="3" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="30" customHeight="1">
@@ -2195,8 +2204,8 @@
       <c r="I10" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="K10" s="3">
-        <v>0</v>
+      <c r="K10" s="3" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="30" customHeight="1">
@@ -2227,8 +2236,8 @@
       <c r="I11" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="K11" s="3">
-        <v>0</v>
+      <c r="K11" s="3" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="30" customHeight="1">
@@ -2355,6 +2364,9 @@
       <c r="I15" s="13" t="s">
         <v>130</v>
       </c>
+      <c r="K15" s="3" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="16" spans="1:11" ht="30" customHeight="1">
       <c r="A16" s="3">
@@ -2480,6 +2492,9 @@
       <c r="I19" s="7" t="s">
         <v>92</v>
       </c>
+      <c r="K19" s="3" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="20" spans="1:11" ht="30" customHeight="1">
       <c r="A20" s="3">
@@ -2509,6 +2524,9 @@
       <c r="I20" s="8" t="s">
         <v>95</v>
       </c>
+      <c r="K20" s="3" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="21" spans="1:11" ht="30" customHeight="1">
       <c r="A21" s="3">
@@ -2538,6 +2556,9 @@
       <c r="I21" s="9" t="s">
         <v>98</v>
       </c>
+      <c r="K21" s="3" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="22" spans="1:11" ht="30" customHeight="1">
       <c r="A22" s="3">
@@ -2631,6 +2652,9 @@
       <c r="I24" s="11" t="s">
         <v>150</v>
       </c>
+      <c r="K24" s="3" t="s">
+        <v>210</v>
+      </c>
     </row>
     <row r="25" spans="1:11" ht="30" customHeight="1">
       <c r="A25" s="3">
@@ -2660,6 +2684,9 @@
       <c r="I25" s="11" t="s">
         <v>152</v>
       </c>
+      <c r="K25" s="3" t="s">
+        <v>211</v>
+      </c>
     </row>
     <row r="26" spans="1:11" ht="30" customHeight="1">
       <c r="A26" s="3">
@@ -2691,6 +2718,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>